<commit_message>
pretrain / non-train data included in grapsh as option and minor fixes
</commit_message>
<xml_diff>
--- a/fermatrica_rep/res/dict/vis_dict.xlsx
+++ b/fermatrica_rep/res/dict/vis_dict.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28129"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28526"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F58FE88-E107-4D75-9836-E65B71913252}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C78B4D54-A573-4974-A7B6-1FFE85931431}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="data" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="768" uniqueCount="543">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="768" uniqueCount="541">
   <si>
     <t>variable</t>
   </si>
@@ -1612,12 +1612,6 @@
     <t>posm</t>
   </si>
   <si>
-    <t>Promotion</t>
-  </si>
-  <si>
-    <t>Промоушн</t>
-  </si>
-  <si>
     <t>pr</t>
   </si>
   <si>
@@ -1636,9 +1630,6 @@
     <t>Tailor Made</t>
   </si>
   <si>
-    <t>На заказ</t>
-  </si>
-  <si>
     <t>PR</t>
   </si>
   <si>
@@ -1649,6 +1640,9 @@
   </si>
   <si>
     <t>Gift Packs</t>
+  </si>
+  <si>
+    <t>POSM</t>
   </si>
 </sst>
 </file>
@@ -2879,7 +2873,7 @@
         <v>526</v>
       </c>
       <c r="D64" t="s">
-        <v>541</v>
+        <v>538</v>
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.25">
@@ -2890,7 +2884,7 @@
         <v>527</v>
       </c>
       <c r="C65" t="s">
-        <v>542</v>
+        <v>539</v>
       </c>
       <c r="D65" t="s">
         <v>528</v>
@@ -2904,10 +2898,10 @@
         <v>529</v>
       </c>
       <c r="C66" t="s">
-        <v>530</v>
+        <v>540</v>
       </c>
       <c r="D66" t="s">
-        <v>531</v>
+        <v>540</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.25">
@@ -2915,13 +2909,13 @@
         <v>43</v>
       </c>
       <c r="B67" s="2" t="s">
-        <v>532</v>
+        <v>530</v>
       </c>
       <c r="C67" t="s">
-        <v>539</v>
+        <v>536</v>
       </c>
       <c r="D67" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.25">
@@ -2929,13 +2923,13 @@
         <v>43</v>
       </c>
       <c r="B68" s="2" t="s">
+        <v>531</v>
+      </c>
+      <c r="C68" t="s">
+        <v>532</v>
+      </c>
+      <c r="D68" t="s">
         <v>533</v>
-      </c>
-      <c r="C68" t="s">
-        <v>534</v>
-      </c>
-      <c r="D68" t="s">
-        <v>535</v>
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.25">
@@ -2943,13 +2937,13 @@
         <v>43</v>
       </c>
       <c r="B69" s="2" t="s">
-        <v>536</v>
+        <v>534</v>
       </c>
       <c r="C69" t="s">
-        <v>537</v>
+        <v>535</v>
       </c>
       <c r="D69" t="s">
-        <v>538</v>
+        <v>535</v>
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.25">

</xml_diff>